<commit_message>
Auto: defensive handling for missing columns in calculo_comissoes.py
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,35 +464,69 @@
           <t>ULTIMA_ATUALIZACAO</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>SALDO_APLICADO</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>99999</v>
+        <v>999999</v>
       </c>
       <c r="B2" t="n">
-        <v>25000</v>
+        <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>45000</v>
+        <v>75</v>
       </c>
       <c r="D2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Realizada</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FATURADO</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2025-10-20T17:25:49.118324</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>-0.75</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>9999991</v>
+      </c>
+      <c r="B3" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Realizada</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>FATURADO</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2025-10-17T17:15:14.850208</t>
-        </is>
-      </c>
+      <c r="C3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-10-20T17:25:49.090067</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Exclusão da aba AUDITORIA e dados completos mostrados em COMISSOES_CALCULADAS
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,38 +495,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2025-10-20T17:25:49.118324</t>
+          <t>2025-10-21T12:09:39.312831</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>-0.75</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>9999991</v>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Nao Realizada</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2025-10-20T17:25:49.090067</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Exclusão da aba AUDITORIA e dados completos mostrados em COMISSOES_CALCULADAS2
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,11 +464,6 @@
           <t>ULTIMA_ATUALIZACAO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>SALDO_APLICADO</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -478,7 +473,7 @@
         <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="D2" t="n">
         <v>0.75</v>
@@ -495,11 +490,8 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2025-10-21T12:09:39.312831</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>-0.75</v>
+          <t>2025-10-21T12:30:36.013043</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Retorno ao último commit de ontem
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -1,84 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m.rafael\Desktop\projetos\Robô para cálculo de comissões 2.0\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578BB05A-B2D6-43F0-B263-27623EBE0D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ESTADO" sheetId="1" r:id="rId1"/>
+    <sheet name="ESTADO" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>PROCESSO</t>
-  </si>
-  <si>
-    <t>VALOR_TOTAL_PROCESSO</t>
-  </si>
-  <si>
-    <t>TOTAL_PAGO_ACUMULADO</t>
-  </si>
-  <si>
-    <t>TOTAL_ADIANTADO_COMISSAO</t>
-  </si>
-  <si>
-    <t>STATUS_PAGAMENTO</t>
-  </si>
-  <si>
-    <t>STATUS_RECONCILIACAO</t>
-  </si>
-  <si>
-    <t>STATUS_PROCESSO_ANALISE</t>
-  </si>
-  <si>
-    <t>ULTIMA_ATUALIZACAO</t>
-  </si>
-  <si>
-    <t>Quitado</t>
-  </si>
-  <si>
-    <t>Realizada</t>
-  </si>
-  <si>
-    <t>FATURADO</t>
-  </si>
-  <si>
-    <t>2025-10-22T17:15:53.040185</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -93,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -417,63 +420,54 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="29.85546875" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>999999</v>
-      </c>
-      <c r="B2">
-        <v>300</v>
-      </c>
-      <c r="C2">
-        <v>325</v>
-      </c>
-      <c r="D2">
-        <v>0.25</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PROCESSO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>VALOR_TOTAL_PROCESSO</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_PAGO_ACUMULADO</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_ADIANTADO_COMISSAO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_PAGAMENTO</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_RECONCILIACAO</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_PROCESSO_ANALISE</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ULTIMA_ATUALIZACAO</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CHECKPOINT ROBÔ COM RECONCILIAÇÕES FUNCIONAL! PEQUENOS BUGS DEVEM SER CORRIGIDOS!
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -1,37 +1,84 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m.rafael\Desktop\projetos\Robô para cálculo de comissões 2.0\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC8A9DF6-3BF4-4ED5-BC6F-9EB9386CD9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ESTADO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ESTADO" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>PROCESSO</t>
+  </si>
+  <si>
+    <t>VALOR_TOTAL_PROCESSO</t>
+  </si>
+  <si>
+    <t>TOTAL_PAGO_ACUMULADO</t>
+  </si>
+  <si>
+    <t>TOTAL_ADIANTADO_COMISSAO</t>
+  </si>
+  <si>
+    <t>STATUS_PAGAMENTO</t>
+  </si>
+  <si>
+    <t>STATUS_RECONCILIACAO</t>
+  </si>
+  <si>
+    <t>STATUS_PROCESSO_ANALISE</t>
+  </si>
+  <si>
+    <t>ULTIMA_ATUALIZACAO</t>
+  </si>
+  <si>
+    <t>Quitado</t>
+  </si>
+  <si>
+    <t>Realizada</t>
+  </si>
+  <si>
+    <t>FATURADO</t>
+  </si>
+  <si>
+    <t>2025-10-23T15:36:24.296816</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +93,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,88 +417,64 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PROCESSO</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>VALOR_TOTAL_PROCESSO</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL_PAGO_ACUMULADO</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL_ADIANTADO_COMISSAO</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS_PAGAMENTO</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS_RECONCILIACAO</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS_PROCESSO_ANALISE</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>ULTIMA_ATUALIZACAO</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>999999</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>300</v>
       </c>
-      <c r="C2" t="n">
-        <v>300</v>
-      </c>
-      <c r="D2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Quitado</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Nao Realizada</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>FATURADO</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2025-10-23T14:28:57.755692</t>
-        </is>
+      <c r="C2">
+        <v>1200</v>
+      </c>
+      <c r="D2">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CHECKPOINT ROBÔ COM RECONCILIAÇÕES FUNCIONAL E PEGANDO SOMENTE O GERENTE DE LINHA CORRETO PARA O CÁLCULO DAS RECONCILIAÇÕES - MELHOR VERSÃO ATÉ A DATA DE 23/10/2025
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -1,84 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m.rafael\Desktop\projetos\Robô para cálculo de comissões 2.0\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC8A9DF6-3BF4-4ED5-BC6F-9EB9386CD9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ESTADO" sheetId="1" r:id="rId1"/>
+    <sheet name="ESTADO" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>PROCESSO</t>
-  </si>
-  <si>
-    <t>VALOR_TOTAL_PROCESSO</t>
-  </si>
-  <si>
-    <t>TOTAL_PAGO_ACUMULADO</t>
-  </si>
-  <si>
-    <t>TOTAL_ADIANTADO_COMISSAO</t>
-  </si>
-  <si>
-    <t>STATUS_PAGAMENTO</t>
-  </si>
-  <si>
-    <t>STATUS_RECONCILIACAO</t>
-  </si>
-  <si>
-    <t>STATUS_PROCESSO_ANALISE</t>
-  </si>
-  <si>
-    <t>ULTIMA_ATUALIZACAO</t>
-  </si>
-  <si>
-    <t>Quitado</t>
-  </si>
-  <si>
-    <t>Realizada</t>
-  </si>
-  <si>
-    <t>FATURADO</t>
-  </si>
-  <si>
-    <t>2025-10-23T15:36:24.296816</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -93,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -417,64 +420,88 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PROCESSO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>VALOR_TOTAL_PROCESSO</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_PAGO_ACUMULADO</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_ADIANTADO_COMISSAO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_PAGAMENTO</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_RECONCILIACAO</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_PROCESSO_ANALISE</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ULTIMA_ATUALIZACAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>999999</v>
+      </c>
+      <c r="B2" t="n">
+        <v>300</v>
+      </c>
+      <c r="C2" t="n">
+        <v>300</v>
+      </c>
+      <c r="D2" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>999999</v>
-      </c>
-      <c r="B2">
-        <v>300</v>
-      </c>
-      <c r="C2">
-        <v>1200</v>
-      </c>
-      <c r="D2">
-        <v>18</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Quitado</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Realizada</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FATURADO</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2025-10-23T17:38:10.086117</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tentativa de simplificar cálculo das comissões de recebimentos e reconciliações - ainda sem funcionar - sem o frontend que estava criando integrado
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -471,11 +471,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>999999</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="C2" t="n">
         <v>325</v>
@@ -483,24 +485,16 @@
       <c r="D2" t="n">
         <v>3.25</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Quitado</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Realizada</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>FATURADO</t>
-        </is>
-      </c>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2025-10-29T01:26:21.364001</t>
+          <t>2025-10-29T23:56:57.455545</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização do frontend feita no trabalho
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,35 +472,139 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>999999</v>
+        <v>209</v>
       </c>
       <c r="B2" t="n">
-        <v>150</v>
+        <v>2586.66</v>
       </c>
       <c r="C2" t="n">
-        <v>325</v>
+        <v>1293.33</v>
       </c>
       <c r="D2" t="n">
-        <v>3.25</v>
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Quitado</t>
+          <t>Em Aberto</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Realizada</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>FATURADO</t>
-        </is>
-      </c>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2025-10-29T01:26:21.364001</t>
+          <t>2025-10-29T11:41:07.428487</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>139157</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2577.89</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2025-10-29T11:41:07.432833</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>141377</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1837.68</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2025-10-29T11:41:07.434986</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1709</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2754.13</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2754.13</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2025-10-29T11:41:07.437565</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>141249</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3390.78</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2025-10-29T11:41:07.441164</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GRANDES MELHORIAS NO FRONTEND
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -481,25 +481,23 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>999999</t>
-        </is>
+      <c r="A2" t="n">
+        <v>999999</v>
       </c>
       <c r="B2" t="n">
         <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="D2" t="n">
-        <v>45513.41</v>
+        <v>182053.64</v>
       </c>
       <c r="E2" t="n">
-        <v>45613.41</v>
+        <v>182453.64</v>
       </c>
       <c r="F2" t="n">
-        <v>456.1341</v>
+        <v>1824.5364</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -518,7 +516,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2025-10-31T11:58:26.173029</t>
+          <t>2025-11-03T16:24:50.928749</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ATUALIZAÇÃO FINAL DO EXPEDIENTE 07/11
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,177 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>STATUS_CALCULO_MEDIAS</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>MES_ANO_FATURAMENTO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>TCMP</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>FCMP</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>ULTIMA_ATUALIZACAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>999998</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 0.010000000000000002}</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 0.0}</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2025-11-07T17:24:44.536077</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 0.010000000000000002}</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 0.0}</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2025-11-07T17:24:44.554518</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CS-Test</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Nao Realizada</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 0.010000000000000002}</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 0.0}</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2025-11-07T17:24:44.580239</t>
         </is>
       </c>
     </row>

</xml_diff>